<commit_message>
n loop spin up close to being ready
</commit_message>
<xml_diff>
--- a/CryoGrid/CryoGridCommunity_results/templates/automatic_loops/NEW_PARAMS.xlsx
+++ b/CryoGrid/CryoGridCommunity_results/templates/automatic_loops/NEW_PARAMS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Utilisateurs\pozsgayv\Documents\CryoGrid_VP_Workflow\CryoGrid\CryoGridCommunity_results\templates\automatic_loops\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DFA99F1-85D4-4EF4-9773-BE20353743F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C4C3C8F-AB71-43D2-94FF-A80AB27B8AB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="20" windowWidth="19180" windowHeight="11260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -139,7 +139,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -155,23 +155,8 @@
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF00CC00"/>
       <name val="Consolas"/>
       <family val="3"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF00B0F0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -194,14 +179,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -214,7 +194,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -532,44 +511,44 @@
   <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.81640625" defaultRowHeight="14.5" outlineLevelRow="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.54296875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="19.54296875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="18.54296875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="16.81640625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="16.453125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="30.54296875" style="2" customWidth="1"/>
-    <col min="7" max="7" width="13.453125" style="2" customWidth="1"/>
-    <col min="8" max="8" width="30.08984375" style="2" customWidth="1"/>
-    <col min="9" max="9" width="21.54296875" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="42.26953125" style="2" customWidth="1"/>
-    <col min="11" max="11" width="9.7265625" style="2" customWidth="1"/>
-    <col min="12" max="12" width="12.1796875" style="2" customWidth="1"/>
-    <col min="13" max="16384" width="8.81640625" style="2"/>
+    <col min="1" max="1" width="23.54296875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="19.54296875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="18.54296875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16.81640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="16.453125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="30.54296875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="13.453125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="30.08984375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="21.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="42.26953125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="9.7265625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="12.1796875" style="1" customWidth="1"/>
+    <col min="13" max="16384" width="8.81640625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B4" s="1">
@@ -577,7 +556,7 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B5" s="1">
@@ -585,7 +564,7 @@
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B6" s="1">
@@ -593,148 +572,145 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="6">
+      <c r="B7" s="3">
         <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="6">
+      <c r="B8" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="7">
+      <c r="B9" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="2">
-        <v>1</v>
-      </c>
-      <c r="C10" s="4"/>
+      <c r="B10" s="1">
+        <v>1</v>
+      </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="8"/>
+      <c r="D11" s="5"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D12" s="8"/>
+      <c r="D12" s="5"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="D13" s="8"/>
+      <c r="D13" s="5"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="D14" s="8"/>
+      <c r="D14" s="5"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B17" s="2">
+      <c r="B17" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B18" s="2">
+      <c r="B18" s="1">
         <v>-2</v>
       </c>
-      <c r="C18" s="9"/>
     </row>
     <row r="19" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35"/>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="D21" s="8"/>
+      <c r="D21" s="5"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="2" t="s">
+      <c r="A23" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="2" t="s">
+      <c r="A24" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="2">
+      <c r="B24" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="2" t="s">
+      <c r="A25" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="26" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="2" t="s">
+      <c r="A26" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A29" s="2" t="s">
+      <c r="A29" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A30" s="2" t="s">
+      <c r="A30" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A31" s="3" t="s">
+      <c r="A31" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B31" s="2">
+      <c r="B31" s="1">
         <v>1</v>
       </c>
     </row>
@@ -747,18 +723,18 @@
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A33" s="2" t="s">
+      <c r="A33" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="B33" s="1" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A34" s="2" t="s">
+      <c r="A34" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C34" s="1">
@@ -770,15 +746,15 @@
       <c r="E34" s="1">
         <v>1</v>
       </c>
-      <c r="F34" s="2" t="s">
+      <c r="F34" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A35" s="2" t="s">
+      <c r="A35" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C35" s="1">
@@ -790,52 +766,52 @@
       <c r="E35" s="1">
         <v>1</v>
       </c>
-      <c r="F35" s="2" t="s">
+      <c r="F35" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A36" s="2" t="s">
+      <c r="A36" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A39" s="2" t="s">
+      <c r="A39" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A40" s="2" t="s">
+      <c r="A40" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="B40" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A41" s="2" t="s">
+      <c r="A41" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B41" s="2">
+      <c r="B41" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A43" s="2" t="s">
+      <c r="A43" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="B43" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D43" s="2" t="s">
+      <c r="D43" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B44" s="2">
+      <c r="B44" s="1">
         <v>0</v>
       </c>
       <c r="C44" s="1">
@@ -851,13 +827,12 @@
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B46" s="2" t="s">
+      <c r="B46" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C46" s="4"/>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A47" s="2" t="s">
+      <c r="A47" s="1" t="s">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Got rid of explicit path names
</commit_message>
<xml_diff>
--- a/CryoGrid/CryoGridCommunity_results/templates/automatic_loops/NEW_PARAMS.xlsx
+++ b/CryoGrid/CryoGridCommunity_results/templates/automatic_loops/NEW_PARAMS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Utilisateurs\pozsgayv\Documents\CryoGrid_VP_Workflow\CryoGrid\CryoGridCommunity_results\templates\automatic_loops\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C4C3C8F-AB71-43D2-94FF-A80AB27B8AB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADDBE8F7-8352-4CE6-B398-495A4F5FB900}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -123,16 +123,16 @@
     <t>horizon_angles</t>
   </si>
   <si>
-    <t>D:\Utilisateurs\pozsgayv\Documents\CryoGrid_VP_Workflow\forcing\Forcing_Data\</t>
-  </si>
-  <si>
     <t>TILE_1D</t>
   </si>
   <si>
     <t>restart_file_path</t>
   </si>
   <si>
-    <t>D:\Utilisateurs\pozsgayv\Documents\CryoGrid_VP_Workflow\CryoGrid\CryoGridCommunity_results\templates\automatic_loops\</t>
+    <t>..\..\forcing\Forcing_Data\</t>
+  </si>
+  <si>
+    <t>..\CryoGridCommunity_results\templates\automatic_loops\</t>
   </si>
 </sst>
 </file>
@@ -636,7 +636,7 @@
     </row>
     <row r="17" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B17" s="1">
         <v>1</v>
@@ -674,7 +674,7 @@
     </row>
     <row r="24" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B24" s="1">
         <v>2</v>
@@ -682,7 +682,7 @@
     </row>
     <row r="25" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>32</v>
@@ -727,7 +727,7 @@
         <v>9</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Fully functioning loop example with restart if broken
</commit_message>
<xml_diff>
--- a/CryoGrid/CryoGridCommunity_results/templates/automatic_loops/NEW_PARAMS.xlsx
+++ b/CryoGrid/CryoGridCommunity_results/templates/automatic_loops/NEW_PARAMS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Utilisateurs\pozsgayv\Documents\CryoGrid_VP_Workflow\CryoGrid\CryoGridCommunity_results\templates\automatic_loops\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41A334B8-AE92-4966-BEE5-023E0F44DAF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B65EDD2E-DEF1-4074-A7F7-7468FBC66CCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -770,7 +770,7 @@
         <v>10</v>
       </c>
       <c r="E28" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>6</v>

</xml_diff>

<commit_message>
Progress with restarting tiles/years within tiles
</commit_message>
<xml_diff>
--- a/CryoGrid/CryoGridCommunity_results/templates/automatic_loops/NEW_PARAMS.xlsx
+++ b/CryoGrid/CryoGridCommunity_results/templates/automatic_loops/NEW_PARAMS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Utilisateurs\pozsgayv\Documents\CryoGrid_VP_Workflow\CryoGrid\CryoGridCommunity_results\templates\automatic_loops\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B65EDD2E-DEF1-4074-A7F7-7468FBC66CCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04B15191-F876-40BE-9BC2-9F4A3254F2E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -747,10 +747,10 @@
         <v>1958</v>
       </c>
       <c r="D27" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E27" s="1">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>6</v>
@@ -764,13 +764,13 @@
         <v>4</v>
       </c>
       <c r="C28" s="1">
-        <v>1958</v>
+        <v>1959</v>
       </c>
       <c r="D28" s="1">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E28" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>6</v>

</xml_diff>